<commit_message>
feat: add DPS Class 6 import script, real roster now in source file
Follow-up to the 2026-07-07 DPS reset — Class 6 was seeded as an empty
shell then because the source file only had placeholder roll numbers.
The owner has since supplied the real 19-student roster.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/School_docs/Daffodils/STUDENTS  INFO. $.xlsx
+++ b/School_docs/Daffodils/STUDENTS  INFO. $.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sxdle\OneDrive\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5988A63-E01F-47CE-B413-D4D3316B5709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2A08202-0B68-486F-90D6-55D027B42951}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FFBB5A24-909C-4739-8B08-CEB770334FA4}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3359" uniqueCount="1174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3835" uniqueCount="1331">
   <si>
     <t>FIRST NAME</t>
   </si>
@@ -3388,9 +3388,6 @@
     <t>08.05.2022</t>
   </si>
   <si>
-    <t>MUSTAG</t>
-  </si>
-  <si>
     <t>ANABIYA</t>
   </si>
   <si>
@@ -3484,9 +3481,6 @@
     <t>09.12.2019</t>
   </si>
   <si>
-    <t xml:space="preserve">DIYANSH </t>
-  </si>
-  <si>
     <t>AARTI</t>
   </si>
   <si>
@@ -3560,6 +3554,483 @@
   </si>
   <si>
     <t>19.02.2022</t>
+  </si>
+  <si>
+    <t>KANISTHA</t>
+  </si>
+  <si>
+    <t>01.09.2015</t>
+  </si>
+  <si>
+    <t>SUNITA ASH</t>
+  </si>
+  <si>
+    <t>DILIP KUMAR ASH</t>
+  </si>
+  <si>
+    <t>27.08.2013</t>
+  </si>
+  <si>
+    <t>TEJAL</t>
+  </si>
+  <si>
+    <t>BABU</t>
+  </si>
+  <si>
+    <t>09.09.2016</t>
+  </si>
+  <si>
+    <t>BISHNU KANT BHAGAT</t>
+  </si>
+  <si>
+    <t>ICHCHA</t>
+  </si>
+  <si>
+    <t>SANGITA DEVI</t>
+  </si>
+  <si>
+    <t>RANTHU MUNDA</t>
+  </si>
+  <si>
+    <t>28.05.2012</t>
+  </si>
+  <si>
+    <t>MD. ALLAUDIN</t>
+  </si>
+  <si>
+    <t>SABRA KHATOON</t>
+  </si>
+  <si>
+    <t>11.08.2014</t>
+  </si>
+  <si>
+    <t>AKHTAR</t>
+  </si>
+  <si>
+    <t>MOIN</t>
+  </si>
+  <si>
+    <t>21.07.2012</t>
+  </si>
+  <si>
+    <t>YOGENDRA MAHTO</t>
+  </si>
+  <si>
+    <t>BABULAL MAHTO</t>
+  </si>
+  <si>
+    <t>18.01.2012</t>
+  </si>
+  <si>
+    <t>AISHA</t>
+  </si>
+  <si>
+    <t>15.12.2015</t>
+  </si>
+  <si>
+    <t>SHRVAN KUMAR</t>
+  </si>
+  <si>
+    <t>DHANESHWAR MAHTO</t>
+  </si>
+  <si>
+    <t>07.04.2014</t>
+  </si>
+  <si>
+    <t>JIVIKA</t>
+  </si>
+  <si>
+    <t>MISTI</t>
+  </si>
+  <si>
+    <t>28.06.2014</t>
+  </si>
+  <si>
+    <t>GOURI DEVI</t>
+  </si>
+  <si>
+    <t>RAJU PANDIT</t>
+  </si>
+  <si>
+    <t>RAJESH RAJAK</t>
+  </si>
+  <si>
+    <t>28.08.2012</t>
+  </si>
+  <si>
+    <t>SONI</t>
+  </si>
+  <si>
+    <t>14.11.2010</t>
+  </si>
+  <si>
+    <t>SABITA DEVI</t>
+  </si>
+  <si>
+    <t>ANU SINGH</t>
+  </si>
+  <si>
+    <t>24.07.2014</t>
+  </si>
+  <si>
+    <t>28.06.2012</t>
+  </si>
+  <si>
+    <t>AMARWATI DEVI</t>
+  </si>
+  <si>
+    <t>RAVI KANT MEHTA</t>
+  </si>
+  <si>
+    <t>REKHA KUKMARI</t>
+  </si>
+  <si>
+    <t>04.07.2015</t>
+  </si>
+  <si>
+    <t>PRINCY</t>
+  </si>
+  <si>
+    <t>08.09.2015</t>
+  </si>
+  <si>
+    <t>SHANY SINGH</t>
+  </si>
+  <si>
+    <t>RUPESH KUMAR</t>
+  </si>
+  <si>
+    <t>AMRITA KAPOOR</t>
+  </si>
+  <si>
+    <t>20.11.2014</t>
+  </si>
+  <si>
+    <t>RANDIP</t>
+  </si>
+  <si>
+    <t>KAPOOR</t>
+  </si>
+  <si>
+    <t>18.05.2015</t>
+  </si>
+  <si>
+    <t>MUSHTAQ</t>
+  </si>
+  <si>
+    <t>DIVYANSH</t>
+  </si>
+  <si>
+    <t>BHARTI</t>
+  </si>
+  <si>
+    <t>PRE. NUR</t>
+  </si>
+  <si>
+    <t>25.09.2022</t>
+  </si>
+  <si>
+    <t>NEHA KUMARI</t>
+  </si>
+  <si>
+    <t>NARESH MAHTO</t>
+  </si>
+  <si>
+    <t>NAYATOLI MESRA, RANCHI</t>
+  </si>
+  <si>
+    <t>31.10.2021</t>
+  </si>
+  <si>
+    <t>RUBY KUMARI</t>
+  </si>
+  <si>
+    <t>MANOJ THAKUR</t>
+  </si>
+  <si>
+    <t>NAMUDAC MANIKA , LATEHAR</t>
+  </si>
+  <si>
+    <t>CHUTTU VIKAS, RANCHI</t>
+  </si>
+  <si>
+    <t>BIRENDRA MUNDA</t>
+  </si>
+  <si>
+    <t>11.11.2022</t>
+  </si>
+  <si>
+    <t>BADAL</t>
+  </si>
+  <si>
+    <t>SURYANSH</t>
+  </si>
+  <si>
+    <t>11.04.2023</t>
+  </si>
+  <si>
+    <t>PUNAM KUMARI</t>
+  </si>
+  <si>
+    <t>YOGENDRA KUMAR MAHTO</t>
+  </si>
+  <si>
+    <t>NEEM TAND BONGAIBERA, RANCHI</t>
+  </si>
+  <si>
+    <t>ROHIT MUNDA</t>
+  </si>
+  <si>
+    <t>KANCHAN KUMARI</t>
+  </si>
+  <si>
+    <t>10.10.2022</t>
+  </si>
+  <si>
+    <t>ADITI</t>
+  </si>
+  <si>
+    <t>SHIVANSH KUMAR</t>
+  </si>
+  <si>
+    <t>05.07.2022</t>
+  </si>
+  <si>
+    <t>JAGESHWAR MAHTO</t>
+  </si>
+  <si>
+    <t>RAJ KISHOR MAHTO</t>
+  </si>
+  <si>
+    <t>GITAN DEVI</t>
+  </si>
+  <si>
+    <t>13.01.2023</t>
+  </si>
+  <si>
+    <t>PRANSHI</t>
+  </si>
+  <si>
+    <t>VIVAN</t>
+  </si>
+  <si>
+    <t>21.08.2022</t>
+  </si>
+  <si>
+    <t>SANJYOTI KUMARI</t>
+  </si>
+  <si>
+    <t>RAJKESHWAR MAHTO</t>
+  </si>
+  <si>
+    <t>CHUTTU, KALI MANDIR MESRA, RANCHI</t>
+  </si>
+  <si>
+    <t>MANESH MAHTO</t>
+  </si>
+  <si>
+    <t>03.03.2023</t>
+  </si>
+  <si>
+    <t>MD. AYSAR</t>
+  </si>
+  <si>
+    <t>28.08.2022</t>
+  </si>
+  <si>
+    <t>MUSTAQ ANSARI</t>
+  </si>
+  <si>
+    <t>CHUTTU NEORI VIKAS</t>
+  </si>
+  <si>
+    <t>05.11.2022</t>
+  </si>
+  <si>
+    <t>NIKKI KUMARI</t>
+  </si>
+  <si>
+    <t>ROHIT KUMAR MAHTO</t>
+  </si>
+  <si>
+    <t>CHUTTU MESRA</t>
+  </si>
+  <si>
+    <t>CHUTTU NEORI MESRA</t>
+  </si>
+  <si>
+    <t>RAKESH KUMAR MAHTO</t>
+  </si>
+  <si>
+    <t>PUNITA KUMARI</t>
+  </si>
+  <si>
+    <t>RIYANSH</t>
+  </si>
+  <si>
+    <t>16.01.2022</t>
+  </si>
+  <si>
+    <t>RESHMA TOPPO</t>
+  </si>
+  <si>
+    <t>SUNIL ORAON</t>
+  </si>
+  <si>
+    <t>AKANSHA</t>
+  </si>
+  <si>
+    <t>ZEBA</t>
+  </si>
+  <si>
+    <t>20.12.2021</t>
+  </si>
+  <si>
+    <t>SHAHNAJ KHATTON</t>
+  </si>
+  <si>
+    <t>CHUTTU MESRA, RANCHI</t>
+  </si>
+  <si>
+    <t>VISHAL MUNDA</t>
+  </si>
+  <si>
+    <t>BINNI KUMARI</t>
+  </si>
+  <si>
+    <t>VEER</t>
+  </si>
+  <si>
+    <t>SINDHU</t>
+  </si>
+  <si>
+    <t>31.12.2022</t>
+  </si>
+  <si>
+    <t>SANJEEV KUMAR MAHTO</t>
+  </si>
+  <si>
+    <t>CHUTTU NEEORI VIKAS</t>
+  </si>
+  <si>
+    <t>TAMESHWAR CHOUDHARY</t>
+  </si>
+  <si>
+    <t>SARITA KUMARI</t>
+  </si>
+  <si>
+    <t>07.07.2023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PRIYA </t>
+  </si>
+  <si>
+    <t>06.03.2022</t>
+  </si>
+  <si>
+    <t>NUSRAT KHATTOON</t>
+  </si>
+  <si>
+    <t>MD. MATAUL ANSARI</t>
+  </si>
+  <si>
+    <t>KABRISTAN , KEDAL</t>
+  </si>
+  <si>
+    <t>JUNGLETOLI MESRA RANCHI</t>
+  </si>
+  <si>
+    <t>RAMESH KUMAR MAHTO</t>
+  </si>
+  <si>
+    <t>SUNITA KUMARI</t>
+  </si>
+  <si>
+    <t>12.05.2023</t>
+  </si>
+  <si>
+    <t>23.10.2023</t>
+  </si>
+  <si>
+    <t>VICKY MAHTO</t>
+  </si>
+  <si>
+    <t>CHUTTU MESRA RANCHI</t>
+  </si>
+  <si>
+    <t>MAHENDRA KUMAR</t>
+  </si>
+  <si>
+    <t>26.05.2023</t>
+  </si>
+  <si>
+    <t>MITHI</t>
+  </si>
+  <si>
+    <t>09.12.2021</t>
+  </si>
+  <si>
+    <t>SUSHMA KUMARI</t>
+  </si>
+  <si>
+    <t>MITHLESH KUMAR SINGH</t>
+  </si>
+  <si>
+    <t>HOMBAI B.I.T MESRA</t>
+  </si>
+  <si>
+    <t>SUNIL LOHRA</t>
+  </si>
+  <si>
+    <t>SUKARMANI KUMARI</t>
+  </si>
+  <si>
+    <t>07.05.2022</t>
+  </si>
+  <si>
+    <t>LOHRA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ABHIRA </t>
+  </si>
+  <si>
+    <t>20.12.2023</t>
+  </si>
+  <si>
+    <t>VIKAS KUMAR SHASHI</t>
+  </si>
+  <si>
+    <t>MESRA NEORI VIKAS</t>
+  </si>
+  <si>
+    <t>MEENU KUMARI</t>
+  </si>
+  <si>
+    <t>12.10.2023</t>
+  </si>
+  <si>
+    <t>11.01.2023</t>
+  </si>
+  <si>
+    <t>ABHIMANYU MAHTO</t>
+  </si>
+  <si>
+    <t>13.04.2022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ARYAN </t>
+  </si>
+  <si>
+    <t>BINA DEVI</t>
+  </si>
+  <si>
+    <t>AJEET KUMAR MAHTO</t>
+  </si>
+  <si>
+    <t>SANGEETA KUMARI</t>
+  </si>
+  <si>
+    <t>15.02.2023</t>
   </si>
 </sst>
 </file>
@@ -5646,6 +6117,12 @@
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
+      <c r="B41" t="s">
+        <v>1172</v>
+      </c>
+      <c r="C41" t="s">
+        <v>15</v>
+      </c>
       <c r="D41">
         <v>6</v>
       </c>
@@ -5654,6 +6131,27 @@
       </c>
       <c r="F41">
         <v>1</v>
+      </c>
+      <c r="G41" t="s">
+        <v>17</v>
+      </c>
+      <c r="H41" t="s">
+        <v>1173</v>
+      </c>
+      <c r="I41" t="s">
+        <v>1174</v>
+      </c>
+      <c r="J41" t="s">
+        <v>1175</v>
+      </c>
+      <c r="K41">
+        <v>7667146201</v>
+      </c>
+      <c r="L41" t="s">
+        <v>21</v>
+      </c>
+      <c r="M41" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="42" spans="1:13">
@@ -5661,6 +6159,12 @@
         <f t="shared" si="0"/>
         <v>41</v>
       </c>
+      <c r="B42" t="s">
+        <v>1177</v>
+      </c>
+      <c r="C42" t="s">
+        <v>15</v>
+      </c>
       <c r="D42">
         <v>6</v>
       </c>
@@ -5669,6 +6173,27 @@
       </c>
       <c r="F42">
         <v>2</v>
+      </c>
+      <c r="G42" t="s">
+        <v>17</v>
+      </c>
+      <c r="H42" t="s">
+        <v>1176</v>
+      </c>
+      <c r="I42" t="s">
+        <v>208</v>
+      </c>
+      <c r="J42" t="s">
+        <v>209</v>
+      </c>
+      <c r="K42">
+        <v>8051034177</v>
+      </c>
+      <c r="L42" t="s">
+        <v>21</v>
+      </c>
+      <c r="M42" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="43" spans="1:13">
@@ -5676,6 +6201,12 @@
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
+      <c r="B43" t="s">
+        <v>212</v>
+      </c>
+      <c r="C43" t="s">
+        <v>1178</v>
+      </c>
       <c r="D43">
         <v>6</v>
       </c>
@@ -5684,6 +6215,27 @@
       </c>
       <c r="F43">
         <v>3</v>
+      </c>
+      <c r="G43" t="s">
+        <v>34</v>
+      </c>
+      <c r="H43" t="s">
+        <v>1179</v>
+      </c>
+      <c r="I43" t="s">
+        <v>852</v>
+      </c>
+      <c r="J43" t="s">
+        <v>1180</v>
+      </c>
+      <c r="K43">
+        <v>9693649545</v>
+      </c>
+      <c r="L43" t="s">
+        <v>21</v>
+      </c>
+      <c r="M43" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="44" spans="1:13">
@@ -5691,6 +6243,12 @@
         <f t="shared" si="0"/>
         <v>43</v>
       </c>
+      <c r="B44" t="s">
+        <v>1181</v>
+      </c>
+      <c r="C44" t="s">
+        <v>15</v>
+      </c>
       <c r="D44">
         <v>6</v>
       </c>
@@ -5699,6 +6257,15 @@
       </c>
       <c r="F44">
         <v>4</v>
+      </c>
+      <c r="G44" t="s">
+        <v>17</v>
+      </c>
+      <c r="L44" t="s">
+        <v>21</v>
+      </c>
+      <c r="M44" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="45" spans="1:13">
@@ -5706,6 +6273,12 @@
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
+      <c r="B45" t="s">
+        <v>357</v>
+      </c>
+      <c r="C45" t="s">
+        <v>33</v>
+      </c>
       <c r="D45">
         <v>6</v>
       </c>
@@ -5714,6 +6287,27 @@
       </c>
       <c r="F45">
         <v>5</v>
+      </c>
+      <c r="G45" t="s">
+        <v>34</v>
+      </c>
+      <c r="H45" t="s">
+        <v>1184</v>
+      </c>
+      <c r="I45" t="s">
+        <v>1182</v>
+      </c>
+      <c r="J45" t="s">
+        <v>1183</v>
+      </c>
+      <c r="K45">
+        <v>9709982344</v>
+      </c>
+      <c r="L45" t="s">
+        <v>21</v>
+      </c>
+      <c r="M45" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="46" spans="1:13">
@@ -5721,6 +6315,12 @@
         <f t="shared" si="0"/>
         <v>45</v>
       </c>
+      <c r="B46" t="s">
+        <v>1189</v>
+      </c>
+      <c r="C46" t="s">
+        <v>1188</v>
+      </c>
       <c r="D46">
         <v>6</v>
       </c>
@@ -5729,6 +6329,27 @@
       </c>
       <c r="F46">
         <v>6</v>
+      </c>
+      <c r="G46" t="s">
+        <v>34</v>
+      </c>
+      <c r="H46" t="s">
+        <v>1187</v>
+      </c>
+      <c r="I46" t="s">
+        <v>1186</v>
+      </c>
+      <c r="J46" t="s">
+        <v>1185</v>
+      </c>
+      <c r="K46">
+        <v>9060404922</v>
+      </c>
+      <c r="L46" t="s">
+        <v>21</v>
+      </c>
+      <c r="M46" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="47" spans="1:13">
@@ -5736,6 +6357,12 @@
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
+      <c r="B47" t="s">
+        <v>91</v>
+      </c>
+      <c r="C47" t="s">
+        <v>76</v>
+      </c>
       <c r="D47">
         <v>6</v>
       </c>
@@ -5744,6 +6371,24 @@
       </c>
       <c r="F47">
         <v>7</v>
+      </c>
+      <c r="G47" t="s">
+        <v>34</v>
+      </c>
+      <c r="H47" t="s">
+        <v>1190</v>
+      </c>
+      <c r="I47" t="s">
+        <v>266</v>
+      </c>
+      <c r="J47" t="s">
+        <v>1191</v>
+      </c>
+      <c r="L47" t="s">
+        <v>21</v>
+      </c>
+      <c r="M47" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="48" spans="1:13">
@@ -5751,6 +6396,12 @@
         <f t="shared" si="0"/>
         <v>47</v>
       </c>
+      <c r="B48" t="s">
+        <v>63</v>
+      </c>
+      <c r="C48" t="s">
+        <v>76</v>
+      </c>
       <c r="D48">
         <v>6</v>
       </c>
@@ -5759,6 +6410,27 @@
       </c>
       <c r="F48">
         <v>8</v>
+      </c>
+      <c r="G48" t="s">
+        <v>34</v>
+      </c>
+      <c r="H48" t="s">
+        <v>1193</v>
+      </c>
+      <c r="I48" t="s">
+        <v>216</v>
+      </c>
+      <c r="J48" t="s">
+        <v>1192</v>
+      </c>
+      <c r="K48">
+        <v>7488968884</v>
+      </c>
+      <c r="L48" t="s">
+        <v>165</v>
+      </c>
+      <c r="M48" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="49" spans="1:13">
@@ -5766,6 +6438,12 @@
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
+      <c r="B49" t="s">
+        <v>1194</v>
+      </c>
+      <c r="C49" t="s">
+        <v>15</v>
+      </c>
       <c r="D49">
         <v>6</v>
       </c>
@@ -5774,6 +6452,27 @@
       </c>
       <c r="F49">
         <v>9</v>
+      </c>
+      <c r="G49" t="s">
+        <v>17</v>
+      </c>
+      <c r="H49" t="s">
+        <v>1195</v>
+      </c>
+      <c r="I49" t="s">
+        <v>789</v>
+      </c>
+      <c r="J49" t="s">
+        <v>1196</v>
+      </c>
+      <c r="K49">
+        <v>9631139453</v>
+      </c>
+      <c r="L49" t="s">
+        <v>21</v>
+      </c>
+      <c r="M49" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="50" spans="1:13">
@@ -5781,6 +6480,12 @@
         <f t="shared" si="0"/>
         <v>49</v>
       </c>
+      <c r="B50" t="s">
+        <v>1199</v>
+      </c>
+      <c r="C50" t="s">
+        <v>15</v>
+      </c>
       <c r="D50">
         <v>6</v>
       </c>
@@ -5789,6 +6494,27 @@
       </c>
       <c r="F50">
         <v>10</v>
+      </c>
+      <c r="G50" t="s">
+        <v>17</v>
+      </c>
+      <c r="H50" t="s">
+        <v>1198</v>
+      </c>
+      <c r="I50" t="s">
+        <v>825</v>
+      </c>
+      <c r="J50" t="s">
+        <v>1197</v>
+      </c>
+      <c r="K50">
+        <v>9263162526</v>
+      </c>
+      <c r="L50" t="s">
+        <v>21</v>
+      </c>
+      <c r="M50" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="51" spans="1:13">
@@ -5796,6 +6522,12 @@
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
+      <c r="B51" t="s">
+        <v>1200</v>
+      </c>
+      <c r="C51" t="s">
+        <v>15</v>
+      </c>
       <c r="D51">
         <v>6</v>
       </c>
@@ -5804,6 +6536,27 @@
       </c>
       <c r="F51">
         <v>11</v>
+      </c>
+      <c r="G51" t="s">
+        <v>17</v>
+      </c>
+      <c r="H51" t="s">
+        <v>1201</v>
+      </c>
+      <c r="I51" t="s">
+        <v>1202</v>
+      </c>
+      <c r="J51" t="s">
+        <v>1203</v>
+      </c>
+      <c r="K51">
+        <v>9199942420</v>
+      </c>
+      <c r="L51" t="s">
+        <v>21</v>
+      </c>
+      <c r="M51" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="52" spans="1:13">
@@ -5811,6 +6564,12 @@
         <f t="shared" si="0"/>
         <v>51</v>
       </c>
+      <c r="B52" t="s">
+        <v>1206</v>
+      </c>
+      <c r="C52" t="s">
+        <v>15</v>
+      </c>
       <c r="D52">
         <v>6</v>
       </c>
@@ -5819,6 +6578,27 @@
       </c>
       <c r="F52">
         <v>12</v>
+      </c>
+      <c r="G52" t="s">
+        <v>17</v>
+      </c>
+      <c r="H52" t="s">
+        <v>1205</v>
+      </c>
+      <c r="I52" t="s">
+        <v>1132</v>
+      </c>
+      <c r="J52" t="s">
+        <v>1204</v>
+      </c>
+      <c r="K52">
+        <v>6207640302</v>
+      </c>
+      <c r="L52" t="s">
+        <v>21</v>
+      </c>
+      <c r="M52" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="53" spans="1:13">
@@ -5826,6 +6606,12 @@
         <f t="shared" si="0"/>
         <v>52</v>
       </c>
+      <c r="B53" t="s">
+        <v>64</v>
+      </c>
+      <c r="C53" t="s">
+        <v>76</v>
+      </c>
       <c r="D53">
         <v>6</v>
       </c>
@@ -5834,6 +6620,27 @@
       </c>
       <c r="F53">
         <v>13</v>
+      </c>
+      <c r="G53" t="s">
+        <v>34</v>
+      </c>
+      <c r="H53" t="s">
+        <v>1207</v>
+      </c>
+      <c r="I53" t="s">
+        <v>1208</v>
+      </c>
+      <c r="J53" t="s">
+        <v>124</v>
+      </c>
+      <c r="K53">
+        <v>9608891304</v>
+      </c>
+      <c r="L53" t="s">
+        <v>165</v>
+      </c>
+      <c r="M53" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="54" spans="1:13">
@@ -5841,6 +6648,12 @@
         <f t="shared" si="0"/>
         <v>53</v>
       </c>
+      <c r="B54" t="s">
+        <v>687</v>
+      </c>
+      <c r="C54" t="s">
+        <v>78</v>
+      </c>
       <c r="D54">
         <v>6</v>
       </c>
@@ -5849,6 +6662,27 @@
       </c>
       <c r="F54">
         <v>14</v>
+      </c>
+      <c r="G54" t="s">
+        <v>34</v>
+      </c>
+      <c r="H54" t="s">
+        <v>1210</v>
+      </c>
+      <c r="I54" t="s">
+        <v>244</v>
+      </c>
+      <c r="J54" t="s">
+        <v>1209</v>
+      </c>
+      <c r="K54">
+        <v>6206814097</v>
+      </c>
+      <c r="L54" t="s">
+        <v>21</v>
+      </c>
+      <c r="M54" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="55" spans="1:13">
@@ -5856,6 +6690,12 @@
         <f t="shared" si="0"/>
         <v>54</v>
       </c>
+      <c r="B55" t="s">
+        <v>32</v>
+      </c>
+      <c r="C55" t="s">
+        <v>492</v>
+      </c>
       <c r="D55">
         <v>6</v>
       </c>
@@ -5864,6 +6704,27 @@
       </c>
       <c r="F55">
         <v>15</v>
+      </c>
+      <c r="G55" t="s">
+        <v>34</v>
+      </c>
+      <c r="H55" t="s">
+        <v>1211</v>
+      </c>
+      <c r="I55" t="s">
+        <v>1212</v>
+      </c>
+      <c r="J55" t="s">
+        <v>581</v>
+      </c>
+      <c r="K55">
+        <v>6299797806</v>
+      </c>
+      <c r="L55" t="s">
+        <v>21</v>
+      </c>
+      <c r="M55" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="56" spans="1:13">
@@ -5871,6 +6732,12 @@
         <f t="shared" si="0"/>
         <v>55</v>
       </c>
+      <c r="B56" t="s">
+        <v>1216</v>
+      </c>
+      <c r="C56" t="s">
+        <v>15</v>
+      </c>
       <c r="D56">
         <v>6</v>
       </c>
@@ -5879,6 +6746,27 @@
       </c>
       <c r="F56">
         <v>16</v>
+      </c>
+      <c r="G56" t="s">
+        <v>17</v>
+      </c>
+      <c r="H56" t="s">
+        <v>1215</v>
+      </c>
+      <c r="I56" t="s">
+        <v>1214</v>
+      </c>
+      <c r="J56" t="s">
+        <v>1213</v>
+      </c>
+      <c r="K56">
+        <v>8271169464</v>
+      </c>
+      <c r="L56" t="s">
+        <v>21</v>
+      </c>
+      <c r="M56" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="57" spans="1:13">
@@ -5886,6 +6774,12 @@
         <f t="shared" si="0"/>
         <v>56</v>
       </c>
+      <c r="B57" t="s">
+        <v>77</v>
+      </c>
+      <c r="C57" t="s">
+        <v>44</v>
+      </c>
       <c r="D57">
         <v>6</v>
       </c>
@@ -5894,6 +6788,27 @@
       </c>
       <c r="F57">
         <v>17</v>
+      </c>
+      <c r="G57" t="s">
+        <v>34</v>
+      </c>
+      <c r="H57" t="s">
+        <v>1217</v>
+      </c>
+      <c r="I57" t="s">
+        <v>558</v>
+      </c>
+      <c r="J57" t="s">
+        <v>1218</v>
+      </c>
+      <c r="K57">
+        <v>7219712772</v>
+      </c>
+      <c r="L57" t="s">
+        <v>21</v>
+      </c>
+      <c r="M57" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="58" spans="1:13">
@@ -5901,6 +6816,12 @@
         <f t="shared" si="0"/>
         <v>57</v>
       </c>
+      <c r="B58" t="s">
+        <v>1222</v>
+      </c>
+      <c r="C58" t="s">
+        <v>1223</v>
+      </c>
       <c r="D58">
         <v>6</v>
       </c>
@@ -5909,6 +6830,27 @@
       </c>
       <c r="F58">
         <v>18</v>
+      </c>
+      <c r="G58" t="s">
+        <v>34</v>
+      </c>
+      <c r="H58" t="s">
+        <v>1221</v>
+      </c>
+      <c r="I58" t="s">
+        <v>1220</v>
+      </c>
+      <c r="J58" t="s">
+        <v>1219</v>
+      </c>
+      <c r="K58">
+        <v>9835053534</v>
+      </c>
+      <c r="L58" t="s">
+        <v>21</v>
+      </c>
+      <c r="M58" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="59" spans="1:13">
@@ -5916,6 +6858,12 @@
         <f t="shared" si="0"/>
         <v>58</v>
       </c>
+      <c r="B59" t="s">
+        <v>104</v>
+      </c>
+      <c r="C59" t="s">
+        <v>15</v>
+      </c>
       <c r="D59">
         <v>6</v>
       </c>
@@ -5924,6 +6872,27 @@
       </c>
       <c r="F59">
         <v>19</v>
+      </c>
+      <c r="G59" t="s">
+        <v>17</v>
+      </c>
+      <c r="H59" t="s">
+        <v>1224</v>
+      </c>
+      <c r="I59" t="s">
+        <v>536</v>
+      </c>
+      <c r="J59" t="s">
+        <v>535</v>
+      </c>
+      <c r="K59">
+        <v>9570209832</v>
+      </c>
+      <c r="L59" t="s">
+        <v>21</v>
+      </c>
+      <c r="M59" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="60" spans="1:13">
@@ -18587,10 +19556,10 @@
         <v>355</v>
       </c>
       <c r="B356" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
       <c r="C356" t="s">
-        <v>1116</v>
+        <v>1225</v>
       </c>
       <c r="D356" t="s">
         <v>1049</v>
@@ -18633,7 +19602,7 @@
         <v>356</v>
       </c>
       <c r="B357" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="C357" t="s">
         <v>76</v>
@@ -18655,10 +19624,10 @@
         <v>1115</v>
       </c>
       <c r="I357" t="s">
+        <v>1118</v>
+      </c>
+      <c r="J357" t="s">
         <v>1119</v>
-      </c>
-      <c r="J357" t="s">
-        <v>1120</v>
       </c>
       <c r="K357">
         <v>9060526715</v>
@@ -18679,7 +19648,7 @@
         <v>357</v>
       </c>
       <c r="B358" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="C358" t="s">
         <v>805</v>
@@ -18698,13 +19667,13 @@
         <v>417</v>
       </c>
       <c r="H358" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="I358" t="s">
         <v>807</v>
       </c>
       <c r="J358" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="K358">
         <v>9934750510</v>
@@ -18725,10 +19694,10 @@
         <v>358</v>
       </c>
       <c r="B359" t="s">
+        <v>1123</v>
+      </c>
+      <c r="C359" t="s">
         <v>1124</v>
-      </c>
-      <c r="C359" t="s">
-        <v>1125</v>
       </c>
       <c r="D359" t="s">
         <v>1049</v>
@@ -18744,13 +19713,13 @@
         <v>417</v>
       </c>
       <c r="H359" t="s">
+        <v>1125</v>
+      </c>
+      <c r="I359" t="s">
         <v>1126</v>
       </c>
-      <c r="I359" t="s">
+      <c r="J359" t="s">
         <v>1127</v>
-      </c>
-      <c r="J359" t="s">
-        <v>1128</v>
       </c>
       <c r="K359">
         <v>6202107462</v>
@@ -18771,7 +19740,7 @@
         <v>359</v>
       </c>
       <c r="B360" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
       <c r="C360" t="s">
         <v>146</v>
@@ -18790,13 +19759,13 @@
         <v>417</v>
       </c>
       <c r="H360" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
       <c r="I360" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
       <c r="J360" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="K360">
         <v>8809418469</v>
@@ -18839,10 +19808,10 @@
         <v>1097</v>
       </c>
       <c r="I361" t="s">
+        <v>1132</v>
+      </c>
+      <c r="J361" t="s">
         <v>1133</v>
-      </c>
-      <c r="J361" t="s">
-        <v>1134</v>
       </c>
       <c r="K361">
         <v>9973542584</v>
@@ -18863,7 +19832,7 @@
         <v>361</v>
       </c>
       <c r="B362" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
       <c r="C362" t="s">
         <v>146</v>
@@ -18882,10 +19851,10 @@
         <v>417</v>
       </c>
       <c r="H362" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="I362" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
       <c r="J362" t="s">
         <v>20</v>
@@ -18928,13 +19897,13 @@
         <v>418</v>
       </c>
       <c r="H363" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="I363" t="s">
         <v>163</v>
       </c>
       <c r="J363" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
       <c r="K363">
         <v>7765836337</v>
@@ -18955,7 +19924,7 @@
         <v>363</v>
       </c>
       <c r="B364" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="C364" t="s">
         <v>78</v>
@@ -18974,7 +19943,7 @@
         <v>417</v>
       </c>
       <c r="H364" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="I364" t="s">
         <v>1084</v>
@@ -19001,7 +19970,7 @@
         <v>364</v>
       </c>
       <c r="B365" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="C365" t="s">
         <v>146</v>
@@ -19020,10 +19989,10 @@
         <v>417</v>
       </c>
       <c r="H365" t="s">
+        <v>1142</v>
+      </c>
+      <c r="I365" t="s">
         <v>1143</v>
-      </c>
-      <c r="I365" t="s">
-        <v>1144</v>
       </c>
       <c r="J365" t="s">
         <v>763</v>
@@ -19066,13 +20035,13 @@
         <v>417</v>
       </c>
       <c r="H366" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="I366" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="J366" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="K366">
         <v>9060512944</v>
@@ -19093,10 +20062,10 @@
         <v>366</v>
       </c>
       <c r="B367" t="s">
-        <v>1148</v>
+        <v>1226</v>
       </c>
       <c r="C367" t="s">
-        <v>1154</v>
+        <v>1152</v>
       </c>
       <c r="D367" t="s">
         <v>1049</v>
@@ -19112,13 +20081,13 @@
         <v>417</v>
       </c>
       <c r="H367" t="s">
-        <v>1168</v>
+        <v>1166</v>
       </c>
       <c r="I367" t="s">
         <v>884</v>
       </c>
       <c r="J367" t="s">
-        <v>1161</v>
+        <v>1159</v>
       </c>
       <c r="K367">
         <v>7004506082</v>
@@ -19130,7 +20099,7 @@
         <v>21</v>
       </c>
       <c r="N367" t="s">
-        <v>1156</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="368" spans="1:14">
@@ -19139,7 +20108,7 @@
         <v>367</v>
       </c>
       <c r="B368" t="s">
-        <v>1149</v>
+        <v>1147</v>
       </c>
       <c r="C368" t="s">
         <v>15</v>
@@ -19158,13 +20127,13 @@
         <v>418</v>
       </c>
       <c r="H368" t="s">
-        <v>1169</v>
+        <v>1167</v>
       </c>
       <c r="I368" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
       <c r="J368" t="s">
-        <v>1162</v>
+        <v>1160</v>
       </c>
       <c r="K368">
         <v>9113125993</v>
@@ -19176,7 +20145,7 @@
         <v>21</v>
       </c>
       <c r="N368" t="s">
-        <v>1157</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="369" spans="1:14">
@@ -19185,7 +20154,7 @@
         <v>368</v>
       </c>
       <c r="B369" t="s">
-        <v>1150</v>
+        <v>1148</v>
       </c>
       <c r="C369" t="s">
         <v>76</v>
@@ -19204,13 +20173,13 @@
         <v>417</v>
       </c>
       <c r="H369" t="s">
-        <v>1170</v>
+        <v>1168</v>
       </c>
       <c r="I369" t="s">
         <v>776</v>
       </c>
       <c r="J369" t="s">
-        <v>1163</v>
+        <v>1161</v>
       </c>
       <c r="K369">
         <v>7004150455</v>
@@ -19222,7 +20191,7 @@
         <v>21</v>
       </c>
       <c r="N369" t="s">
-        <v>1158</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="370" spans="1:14">
@@ -19231,7 +20200,7 @@
         <v>369</v>
       </c>
       <c r="B370" t="s">
-        <v>1151</v>
+        <v>1149</v>
       </c>
       <c r="C370" t="s">
         <v>293</v>
@@ -19250,13 +20219,13 @@
         <v>418</v>
       </c>
       <c r="H370" t="s">
-        <v>1171</v>
+        <v>1169</v>
       </c>
       <c r="I370" t="s">
         <v>869</v>
       </c>
       <c r="J370" t="s">
-        <v>1164</v>
+        <v>1162</v>
       </c>
       <c r="K370">
         <v>9472770967</v>
@@ -19268,7 +20237,7 @@
         <v>21</v>
       </c>
       <c r="N370" t="s">
-        <v>1159</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="371" spans="1:14">
@@ -19277,7 +20246,7 @@
         <v>370</v>
       </c>
       <c r="B371" t="s">
-        <v>1152</v>
+        <v>1150</v>
       </c>
       <c r="C371" t="s">
         <v>87</v>
@@ -19296,13 +20265,13 @@
         <v>417</v>
       </c>
       <c r="H371" t="s">
-        <v>1172</v>
+        <v>1170</v>
       </c>
       <c r="I371" t="s">
         <v>226</v>
       </c>
       <c r="J371" t="s">
-        <v>1165</v>
+        <v>1163</v>
       </c>
       <c r="K371">
         <v>8084638833</v>
@@ -19323,10 +20292,10 @@
         <v>371</v>
       </c>
       <c r="B372" t="s">
+        <v>1151</v>
+      </c>
+      <c r="C372" t="s">
         <v>1153</v>
-      </c>
-      <c r="C372" t="s">
-        <v>1155</v>
       </c>
       <c r="D372" t="s">
         <v>1049</v>
@@ -19342,13 +20311,13 @@
         <v>418</v>
       </c>
       <c r="H372" t="s">
-        <v>1173</v>
+        <v>1171</v>
       </c>
       <c r="I372" t="s">
-        <v>1167</v>
+        <v>1165</v>
       </c>
       <c r="J372" t="s">
-        <v>1166</v>
+        <v>1164</v>
       </c>
       <c r="L372" t="s">
         <v>165</v>
@@ -19357,7 +20326,7 @@
         <v>21</v>
       </c>
       <c r="N372" t="s">
-        <v>1160</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="373" spans="1:14">
@@ -19365,400 +20334,1590 @@
         <f t="shared" si="12"/>
         <v>372</v>
       </c>
+      <c r="B373" t="s">
+        <v>184</v>
+      </c>
+      <c r="C373" t="s">
+        <v>1227</v>
+      </c>
+      <c r="D373" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E373" t="s">
+        <v>16</v>
+      </c>
+      <c r="F373">
+        <v>1</v>
+      </c>
+      <c r="G373" t="s">
+        <v>418</v>
+      </c>
+      <c r="H373" t="s">
+        <v>1229</v>
+      </c>
+      <c r="I373" t="s">
+        <v>1230</v>
+      </c>
+      <c r="J373" t="s">
+        <v>1231</v>
+      </c>
+      <c r="K373">
+        <v>9608886663</v>
+      </c>
+      <c r="L373" t="s">
+        <v>21</v>
+      </c>
+      <c r="M373" t="s">
+        <v>21</v>
+      </c>
+      <c r="N373" t="s">
+        <v>1232</v>
+      </c>
     </row>
     <row r="374" spans="1:14">
       <c r="A374">
         <f t="shared" si="12"/>
         <v>373</v>
       </c>
+      <c r="B374" t="s">
+        <v>1092</v>
+      </c>
+      <c r="C374" t="s">
+        <v>76</v>
+      </c>
+      <c r="D374" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E374" t="s">
+        <v>16</v>
+      </c>
+      <c r="F374">
+        <f>1+F373</f>
+        <v>2</v>
+      </c>
+      <c r="G374" t="s">
+        <v>417</v>
+      </c>
+      <c r="H374" t="s">
+        <v>1233</v>
+      </c>
+      <c r="I374" t="s">
+        <v>1234</v>
+      </c>
+      <c r="J374" t="s">
+        <v>1235</v>
+      </c>
+      <c r="K374">
+        <v>7667789396</v>
+      </c>
+      <c r="L374" t="s">
+        <v>165</v>
+      </c>
+      <c r="M374" t="s">
+        <v>21</v>
+      </c>
+      <c r="N374" t="s">
+        <v>1236</v>
+      </c>
     </row>
     <row r="375" spans="1:14">
       <c r="A375">
         <f t="shared" si="12"/>
         <v>374</v>
       </c>
+      <c r="B375" t="s">
+        <v>1240</v>
+      </c>
+      <c r="C375" t="s">
+        <v>33</v>
+      </c>
+      <c r="D375" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E375" t="s">
+        <v>16</v>
+      </c>
+      <c r="F375">
+        <f t="shared" ref="F375:F409" si="14">1+F374</f>
+        <v>3</v>
+      </c>
+      <c r="G375" t="s">
+        <v>417</v>
+      </c>
+      <c r="H375" t="s">
+        <v>1239</v>
+      </c>
+      <c r="I375" t="s">
+        <v>807</v>
+      </c>
+      <c r="J375" t="s">
+        <v>1238</v>
+      </c>
+      <c r="K375">
+        <v>8709362822</v>
+      </c>
+      <c r="L375" t="s">
+        <v>21</v>
+      </c>
+      <c r="M375" t="s">
+        <v>21</v>
+      </c>
+      <c r="N375" t="s">
+        <v>1237</v>
+      </c>
     </row>
     <row r="376" spans="1:14">
       <c r="A376">
         <f t="shared" si="12"/>
         <v>375</v>
       </c>
+      <c r="B376" t="s">
+        <v>1241</v>
+      </c>
+      <c r="C376" t="s">
+        <v>76</v>
+      </c>
+      <c r="D376" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E376" t="s">
+        <v>16</v>
+      </c>
+      <c r="F376">
+        <f t="shared" si="14"/>
+        <v>4</v>
+      </c>
+      <c r="G376" t="s">
+        <v>417</v>
+      </c>
+      <c r="H376" t="s">
+        <v>1242</v>
+      </c>
+      <c r="I376" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J376" t="s">
+        <v>1244</v>
+      </c>
+      <c r="K376">
+        <v>7250764829</v>
+      </c>
+      <c r="L376" t="s">
+        <v>21</v>
+      </c>
+      <c r="M376" t="s">
+        <v>21</v>
+      </c>
+      <c r="N376" t="s">
+        <v>425</v>
+      </c>
     </row>
     <row r="377" spans="1:14">
       <c r="A377">
         <f t="shared" si="12"/>
         <v>376</v>
       </c>
+      <c r="B377" t="s">
+        <v>1249</v>
+      </c>
+      <c r="C377" t="s">
+        <v>33</v>
+      </c>
+      <c r="D377" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E377" t="s">
+        <v>16</v>
+      </c>
+      <c r="F377">
+        <f t="shared" si="14"/>
+        <v>5</v>
+      </c>
+      <c r="G377" t="s">
+        <v>418</v>
+      </c>
+      <c r="H377" t="s">
+        <v>1248</v>
+      </c>
+      <c r="I377" t="s">
+        <v>1247</v>
+      </c>
+      <c r="J377" t="s">
+        <v>1246</v>
+      </c>
+      <c r="K377">
+        <v>9572208234</v>
+      </c>
+      <c r="L377" t="s">
+        <v>21</v>
+      </c>
+      <c r="M377" t="s">
+        <v>21</v>
+      </c>
+      <c r="N377" t="s">
+        <v>1245</v>
+      </c>
     </row>
     <row r="378" spans="1:14">
       <c r="A378">
         <f t="shared" si="12"/>
         <v>377</v>
       </c>
+      <c r="B378" t="s">
+        <v>1250</v>
+      </c>
+      <c r="C378" t="s">
+        <v>146</v>
+      </c>
+      <c r="D378" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E378" t="s">
+        <v>16</v>
+      </c>
+      <c r="F378">
+        <f t="shared" si="14"/>
+        <v>6</v>
+      </c>
+      <c r="G378" t="s">
+        <v>417</v>
+      </c>
+      <c r="H378" t="s">
+        <v>1251</v>
+      </c>
+      <c r="I378" t="s">
+        <v>628</v>
+      </c>
+      <c r="J378" t="s">
+        <v>1252</v>
+      </c>
+      <c r="K378">
+        <v>8709104670</v>
+      </c>
+      <c r="L378" t="s">
+        <v>21</v>
+      </c>
+      <c r="M378" t="s">
+        <v>21</v>
+      </c>
+      <c r="N378" t="s">
+        <v>425</v>
+      </c>
     </row>
     <row r="379" spans="1:14">
       <c r="A379">
         <f t="shared" si="12"/>
         <v>378</v>
       </c>
+      <c r="B379" t="s">
+        <v>1256</v>
+      </c>
+      <c r="C379" t="s">
+        <v>15</v>
+      </c>
+      <c r="D379" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E379" t="s">
+        <v>16</v>
+      </c>
+      <c r="F379">
+        <f t="shared" si="14"/>
+        <v>7</v>
+      </c>
+      <c r="G379" t="s">
+        <v>418</v>
+      </c>
+      <c r="H379" t="s">
+        <v>1255</v>
+      </c>
+      <c r="I379" t="s">
+        <v>1254</v>
+      </c>
+      <c r="J379" t="s">
+        <v>1253</v>
+      </c>
+      <c r="K379">
+        <v>9122447650</v>
+      </c>
+      <c r="L379" t="s">
+        <v>21</v>
+      </c>
+      <c r="M379" t="s">
+        <v>21</v>
+      </c>
+      <c r="N379" t="s">
+        <v>425</v>
+      </c>
     </row>
     <row r="380" spans="1:14">
       <c r="A380">
         <f t="shared" si="12"/>
         <v>379</v>
       </c>
+      <c r="B380" t="s">
+        <v>1257</v>
+      </c>
+      <c r="C380" t="s">
+        <v>146</v>
+      </c>
+      <c r="D380" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E380" t="s">
+        <v>16</v>
+      </c>
+      <c r="F380">
+        <f t="shared" si="14"/>
+        <v>8</v>
+      </c>
+      <c r="G380" t="s">
+        <v>417</v>
+      </c>
+      <c r="H380" t="s">
+        <v>1258</v>
+      </c>
+      <c r="I380" t="s">
+        <v>1259</v>
+      </c>
+      <c r="J380" t="s">
+        <v>1260</v>
+      </c>
+      <c r="K380">
+        <v>8210225982</v>
+      </c>
+      <c r="L380" t="s">
+        <v>21</v>
+      </c>
+      <c r="M380" t="s">
+        <v>21</v>
+      </c>
+      <c r="N380" t="s">
+        <v>1261</v>
+      </c>
     </row>
     <row r="381" spans="1:14">
       <c r="A381">
         <f t="shared" si="12"/>
         <v>380</v>
       </c>
+      <c r="B381" t="s">
+        <v>1103</v>
+      </c>
+      <c r="C381" t="s">
+        <v>15</v>
+      </c>
+      <c r="D381" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E381" t="s">
+        <v>16</v>
+      </c>
+      <c r="F381">
+        <f t="shared" si="14"/>
+        <v>9</v>
+      </c>
+      <c r="G381" t="s">
+        <v>418</v>
+      </c>
+      <c r="H381" t="s">
+        <v>1263</v>
+      </c>
+      <c r="I381" t="s">
+        <v>869</v>
+      </c>
+      <c r="J381" t="s">
+        <v>1262</v>
+      </c>
+      <c r="K381">
+        <v>9608576844</v>
+      </c>
+      <c r="L381" t="s">
+        <v>21</v>
+      </c>
+      <c r="M381" t="s">
+        <v>21</v>
+      </c>
+      <c r="N381" t="s">
+        <v>425</v>
+      </c>
     </row>
     <row r="382" spans="1:14">
       <c r="A382">
         <f t="shared" si="12"/>
         <v>381</v>
       </c>
+      <c r="B382" t="s">
+        <v>1264</v>
+      </c>
+      <c r="D382" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E382" t="s">
+        <v>16</v>
+      </c>
+      <c r="F382">
+        <f t="shared" si="14"/>
+        <v>10</v>
+      </c>
+      <c r="G382" t="s">
+        <v>417</v>
+      </c>
+      <c r="H382" t="s">
+        <v>1265</v>
+      </c>
+      <c r="I382" t="s">
+        <v>1114</v>
+      </c>
+      <c r="J382" t="s">
+        <v>1266</v>
+      </c>
+      <c r="K382">
+        <v>8051086380</v>
+      </c>
+      <c r="L382" t="s">
+        <v>21</v>
+      </c>
+      <c r="M382" t="s">
+        <v>21</v>
+      </c>
+      <c r="N382" t="s">
+        <v>1267</v>
+      </c>
     </row>
     <row r="383" spans="1:14">
       <c r="A383">
         <f t="shared" si="12"/>
         <v>382</v>
       </c>
+      <c r="B383" t="s">
+        <v>1226</v>
+      </c>
+      <c r="C383" t="s">
+        <v>76</v>
+      </c>
+      <c r="D383" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E383" t="s">
+        <v>16</v>
+      </c>
+      <c r="F383">
+        <f t="shared" si="14"/>
+        <v>11</v>
+      </c>
+      <c r="G383" t="s">
+        <v>417</v>
+      </c>
+      <c r="H383" t="s">
+        <v>1268</v>
+      </c>
+      <c r="I383" t="s">
+        <v>1269</v>
+      </c>
+      <c r="J383" t="s">
+        <v>1270</v>
+      </c>
+      <c r="K383">
+        <v>6201157306</v>
+      </c>
+      <c r="L383" t="s">
+        <v>21</v>
+      </c>
+      <c r="M383" t="s">
+        <v>21</v>
+      </c>
+      <c r="N383" t="s">
+        <v>1271</v>
+      </c>
     </row>
     <row r="384" spans="1:14">
       <c r="A384">
         <f t="shared" si="12"/>
         <v>383</v>
       </c>
-    </row>
-    <row r="385" spans="1:1">
+      <c r="B384" t="s">
+        <v>419</v>
+      </c>
+      <c r="C384" t="s">
+        <v>146</v>
+      </c>
+      <c r="D384" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E384" t="s">
+        <v>16</v>
+      </c>
+      <c r="F384">
+        <f t="shared" si="14"/>
+        <v>12</v>
+      </c>
+      <c r="G384" t="s">
+        <v>418</v>
+      </c>
+      <c r="H384" t="s">
+        <v>1229</v>
+      </c>
+      <c r="I384" t="s">
+        <v>1274</v>
+      </c>
+      <c r="J384" t="s">
+        <v>1273</v>
+      </c>
+      <c r="K384">
+        <v>8252095212</v>
+      </c>
+      <c r="L384" t="s">
+        <v>21</v>
+      </c>
+      <c r="M384" t="s">
+        <v>21</v>
+      </c>
+      <c r="N384" t="s">
+        <v>1272</v>
+      </c>
+    </row>
+    <row r="385" spans="1:14">
       <c r="A385">
         <f t="shared" si="12"/>
         <v>384</v>
       </c>
-    </row>
-    <row r="386" spans="1:1">
+      <c r="B385" t="s">
+        <v>1275</v>
+      </c>
+      <c r="C385" t="s">
+        <v>293</v>
+      </c>
+      <c r="D385" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E385" t="s">
+        <v>16</v>
+      </c>
+      <c r="F385">
+        <f t="shared" si="14"/>
+        <v>13</v>
+      </c>
+      <c r="G385" t="s">
+        <v>417</v>
+      </c>
+      <c r="H385" t="s">
+        <v>1276</v>
+      </c>
+      <c r="I385" t="s">
+        <v>1277</v>
+      </c>
+      <c r="J385" t="s">
+        <v>1278</v>
+      </c>
+      <c r="K385">
+        <v>6201342657</v>
+      </c>
+      <c r="L385" t="s">
+        <v>165</v>
+      </c>
+      <c r="M385" t="s">
+        <v>21</v>
+      </c>
+      <c r="N385" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="386" spans="1:14">
       <c r="A386">
         <f t="shared" si="12"/>
         <v>385</v>
       </c>
-    </row>
-    <row r="387" spans="1:1">
+      <c r="B386" t="s">
+        <v>1279</v>
+      </c>
+      <c r="C386" t="s">
+        <v>29</v>
+      </c>
+      <c r="D386" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E386" t="s">
+        <v>16</v>
+      </c>
+      <c r="F386">
+        <f t="shared" si="14"/>
+        <v>14</v>
+      </c>
+      <c r="G386" t="s">
+        <v>418</v>
+      </c>
+      <c r="H386" t="s">
+        <v>1040</v>
+      </c>
+      <c r="I386" t="s">
+        <v>697</v>
+      </c>
+      <c r="J386" t="s">
+        <v>696</v>
+      </c>
+      <c r="K386">
+        <v>9304929212</v>
+      </c>
+      <c r="L386" t="s">
+        <v>165</v>
+      </c>
+      <c r="M386" t="s">
+        <v>21</v>
+      </c>
+      <c r="N386" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="387" spans="1:14">
       <c r="A387">
         <f t="shared" si="12"/>
         <v>386</v>
       </c>
-    </row>
-    <row r="388" spans="1:1">
+      <c r="B387" t="s">
+        <v>1280</v>
+      </c>
+      <c r="C387" t="s">
+        <v>560</v>
+      </c>
+      <c r="D387" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E387" t="s">
+        <v>16</v>
+      </c>
+      <c r="F387">
+        <f t="shared" si="14"/>
+        <v>15</v>
+      </c>
+      <c r="G387" t="s">
+        <v>418</v>
+      </c>
+      <c r="H387" t="s">
+        <v>1281</v>
+      </c>
+      <c r="I387" t="s">
+        <v>1282</v>
+      </c>
+      <c r="J387" t="s">
+        <v>778</v>
+      </c>
+      <c r="K387">
+        <v>9113442540</v>
+      </c>
+      <c r="L387" t="s">
+        <v>165</v>
+      </c>
+      <c r="M387" t="s">
+        <v>21</v>
+      </c>
+      <c r="N387" t="s">
+        <v>1283</v>
+      </c>
+    </row>
+    <row r="388" spans="1:14">
       <c r="A388">
         <f t="shared" si="12"/>
         <v>387</v>
       </c>
-    </row>
-    <row r="389" spans="1:1">
+      <c r="B388" t="s">
+        <v>1286</v>
+      </c>
+      <c r="C388" t="s">
+        <v>33</v>
+      </c>
+      <c r="D388" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E388" t="s">
+        <v>16</v>
+      </c>
+      <c r="F388">
+        <f t="shared" si="14"/>
+        <v>16</v>
+      </c>
+      <c r="G388" t="s">
+        <v>417</v>
+      </c>
+      <c r="H388" t="s">
+        <v>1110</v>
+      </c>
+      <c r="I388" t="s">
+        <v>1285</v>
+      </c>
+      <c r="J388" t="s">
+        <v>1284</v>
+      </c>
+      <c r="K388">
+        <v>9905196575</v>
+      </c>
+      <c r="L388" t="s">
+        <v>21</v>
+      </c>
+      <c r="M388" t="s">
+        <v>21</v>
+      </c>
+      <c r="N388" t="s">
+        <v>992</v>
+      </c>
+    </row>
+    <row r="389" spans="1:14">
       <c r="A389">
-        <f t="shared" ref="A389:A439" si="14">1+A388</f>
+        <f t="shared" ref="A389:A439" si="15">1+A388</f>
         <v>388</v>
       </c>
-    </row>
-    <row r="390" spans="1:1">
+      <c r="B389" t="s">
+        <v>1287</v>
+      </c>
+      <c r="C389" t="s">
+        <v>15</v>
+      </c>
+      <c r="D389" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E389" t="s">
+        <v>16</v>
+      </c>
+      <c r="F389">
+        <f t="shared" si="14"/>
+        <v>17</v>
+      </c>
+      <c r="G389" t="s">
+        <v>418</v>
+      </c>
+      <c r="H389" t="s">
+        <v>1288</v>
+      </c>
+      <c r="I389" t="s">
+        <v>252</v>
+      </c>
+      <c r="J389" t="s">
+        <v>1289</v>
+      </c>
+      <c r="K389">
+        <v>7479887474</v>
+      </c>
+      <c r="L389" t="s">
+        <v>21</v>
+      </c>
+      <c r="M389" t="s">
+        <v>21</v>
+      </c>
+      <c r="N389" t="s">
+        <v>1290</v>
+      </c>
+    </row>
+    <row r="390" spans="1:14">
       <c r="A390">
+        <f t="shared" si="15"/>
+        <v>389</v>
+      </c>
+      <c r="B390" t="s">
+        <v>1294</v>
+      </c>
+      <c r="C390" t="s">
+        <v>15</v>
+      </c>
+      <c r="D390" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E390" t="s">
+        <v>16</v>
+      </c>
+      <c r="F390">
         <f t="shared" si="14"/>
-        <v>389</v>
-      </c>
-    </row>
-    <row r="391" spans="1:1">
+        <v>18</v>
+      </c>
+      <c r="G390" t="s">
+        <v>418</v>
+      </c>
+      <c r="H390" t="s">
+        <v>1293</v>
+      </c>
+      <c r="I390" t="s">
+        <v>1292</v>
+      </c>
+      <c r="J390" t="s">
+        <v>1291</v>
+      </c>
+      <c r="K390">
+        <v>7808214466</v>
+      </c>
+      <c r="L390" t="s">
+        <v>21</v>
+      </c>
+      <c r="M390" t="s">
+        <v>21</v>
+      </c>
+      <c r="N390" t="s">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="391" spans="1:14">
       <c r="A391">
+        <f t="shared" si="15"/>
+        <v>390</v>
+      </c>
+      <c r="B391" t="s">
+        <v>14</v>
+      </c>
+      <c r="C391" t="s">
+        <v>137</v>
+      </c>
+      <c r="D391" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E391" t="s">
+        <v>16</v>
+      </c>
+      <c r="F391">
         <f t="shared" si="14"/>
-        <v>390</v>
-      </c>
-    </row>
-    <row r="392" spans="1:1">
+        <v>19</v>
+      </c>
+      <c r="G391" t="s">
+        <v>418</v>
+      </c>
+      <c r="H391" t="s">
+        <v>1295</v>
+      </c>
+      <c r="I391" t="s">
+        <v>1296</v>
+      </c>
+      <c r="J391" t="s">
+        <v>1297</v>
+      </c>
+      <c r="K391">
+        <v>9709014313</v>
+      </c>
+      <c r="L391" t="s">
+        <v>165</v>
+      </c>
+      <c r="M391" t="s">
+        <v>21</v>
+      </c>
+      <c r="N391" t="s">
+        <v>1298</v>
+      </c>
+    </row>
+    <row r="392" spans="1:14">
       <c r="A392">
+        <f t="shared" si="15"/>
+        <v>391</v>
+      </c>
+      <c r="B392" t="s">
+        <v>14</v>
+      </c>
+      <c r="C392" t="s">
+        <v>15</v>
+      </c>
+      <c r="D392" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E392" t="s">
+        <v>16</v>
+      </c>
+      <c r="F392">
         <f t="shared" si="14"/>
-        <v>391</v>
-      </c>
-    </row>
-    <row r="393" spans="1:1">
+        <v>20</v>
+      </c>
+      <c r="G392" t="s">
+        <v>418</v>
+      </c>
+      <c r="H392" t="s">
+        <v>1302</v>
+      </c>
+      <c r="I392" t="s">
+        <v>1301</v>
+      </c>
+      <c r="J392" t="s">
+        <v>1300</v>
+      </c>
+      <c r="K392">
+        <v>9570770879</v>
+      </c>
+      <c r="L392" t="s">
+        <v>165</v>
+      </c>
+      <c r="M392" t="s">
+        <v>21</v>
+      </c>
+      <c r="N392" t="s">
+        <v>1299</v>
+      </c>
+    </row>
+    <row r="393" spans="1:14">
       <c r="A393">
+        <f t="shared" si="15"/>
+        <v>392</v>
+      </c>
+      <c r="B393" t="s">
+        <v>1199</v>
+      </c>
+      <c r="C393" t="s">
+        <v>15</v>
+      </c>
+      <c r="D393" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E393" t="s">
+        <v>16</v>
+      </c>
+      <c r="F393">
         <f t="shared" si="14"/>
-        <v>392</v>
-      </c>
-    </row>
-    <row r="394" spans="1:1">
+        <v>21</v>
+      </c>
+      <c r="G393" t="s">
+        <v>418</v>
+      </c>
+      <c r="H393" t="s">
+        <v>1303</v>
+      </c>
+      <c r="I393" t="s">
+        <v>960</v>
+      </c>
+      <c r="J393" t="s">
+        <v>1304</v>
+      </c>
+      <c r="K393">
+        <v>9122181028</v>
+      </c>
+      <c r="L393" t="s">
+        <v>21</v>
+      </c>
+      <c r="M393" t="s">
+        <v>21</v>
+      </c>
+      <c r="N393" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="394" spans="1:14">
       <c r="A394">
+        <f t="shared" si="15"/>
+        <v>393</v>
+      </c>
+      <c r="B394" t="s">
+        <v>82</v>
+      </c>
+      <c r="C394" t="s">
+        <v>76</v>
+      </c>
+      <c r="D394" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E394" t="s">
+        <v>16</v>
+      </c>
+      <c r="F394">
         <f t="shared" si="14"/>
-        <v>393</v>
-      </c>
-    </row>
-    <row r="395" spans="1:1">
+        <v>22</v>
+      </c>
+      <c r="G394" t="s">
+        <v>417</v>
+      </c>
+      <c r="H394" t="s">
+        <v>1307</v>
+      </c>
+      <c r="I394" t="s">
+        <v>473</v>
+      </c>
+      <c r="J394" t="s">
+        <v>1306</v>
+      </c>
+      <c r="K394">
+        <v>8084002966</v>
+      </c>
+      <c r="L394" t="s">
+        <v>21</v>
+      </c>
+      <c r="M394" t="s">
+        <v>21</v>
+      </c>
+      <c r="N394" t="s">
+        <v>1305</v>
+      </c>
+    </row>
+    <row r="395" spans="1:14">
       <c r="A395">
+        <f t="shared" si="15"/>
+        <v>394</v>
+      </c>
+      <c r="B395" t="s">
+        <v>1308</v>
+      </c>
+      <c r="C395" t="s">
+        <v>15</v>
+      </c>
+      <c r="D395" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E395" t="s">
+        <v>16</v>
+      </c>
+      <c r="F395">
         <f t="shared" si="14"/>
-        <v>394</v>
-      </c>
-    </row>
-    <row r="396" spans="1:1">
+        <v>23</v>
+      </c>
+      <c r="G395" t="s">
+        <v>418</v>
+      </c>
+      <c r="H395" t="s">
+        <v>1309</v>
+      </c>
+      <c r="I395" t="s">
+        <v>1310</v>
+      </c>
+      <c r="J395" t="s">
+        <v>1311</v>
+      </c>
+      <c r="K395">
+        <v>8877148663</v>
+      </c>
+      <c r="L395" t="s">
+        <v>165</v>
+      </c>
+      <c r="M395" t="s">
+        <v>21</v>
+      </c>
+      <c r="N395" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="396" spans="1:14">
       <c r="A396">
+        <f t="shared" si="15"/>
+        <v>395</v>
+      </c>
+      <c r="B396" t="s">
+        <v>519</v>
+      </c>
+      <c r="C396" t="s">
+        <v>1316</v>
+      </c>
+      <c r="D396" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E396" t="s">
+        <v>16</v>
+      </c>
+      <c r="F396">
         <f t="shared" si="14"/>
-        <v>395</v>
-      </c>
-    </row>
-    <row r="397" spans="1:1">
+        <v>24</v>
+      </c>
+      <c r="G396" t="s">
+        <v>417</v>
+      </c>
+      <c r="H396" t="s">
+        <v>1315</v>
+      </c>
+      <c r="I396" t="s">
+        <v>1314</v>
+      </c>
+      <c r="J396" t="s">
+        <v>1313</v>
+      </c>
+      <c r="K396">
+        <v>9608485682</v>
+      </c>
+      <c r="L396" t="s">
+        <v>165</v>
+      </c>
+      <c r="M396" t="s">
+        <v>21</v>
+      </c>
+      <c r="N396" t="s">
+        <v>1312</v>
+      </c>
+    </row>
+    <row r="397" spans="1:14">
       <c r="A397">
+        <f t="shared" si="15"/>
+        <v>396</v>
+      </c>
+      <c r="B397" t="s">
+        <v>1317</v>
+      </c>
+      <c r="C397" t="s">
+        <v>146</v>
+      </c>
+      <c r="D397" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E397" t="s">
+        <v>16</v>
+      </c>
+      <c r="F397">
         <f t="shared" si="14"/>
-        <v>396</v>
-      </c>
-    </row>
-    <row r="398" spans="1:1">
+        <v>25</v>
+      </c>
+      <c r="G397" t="s">
+        <v>418</v>
+      </c>
+      <c r="H397" t="s">
+        <v>1318</v>
+      </c>
+      <c r="I397" t="s">
+        <v>1319</v>
+      </c>
+      <c r="J397" t="s">
+        <v>1145</v>
+      </c>
+      <c r="K397">
+        <v>8252885856</v>
+      </c>
+      <c r="L397" t="s">
+        <v>21</v>
+      </c>
+      <c r="M397" t="s">
+        <v>21</v>
+      </c>
+      <c r="N397" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="398" spans="1:14">
       <c r="A398">
+        <f t="shared" si="15"/>
+        <v>397</v>
+      </c>
+      <c r="B398" t="s">
+        <v>1249</v>
+      </c>
+      <c r="C398" t="s">
+        <v>146</v>
+      </c>
+      <c r="D398" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E398" t="s">
+        <v>16</v>
+      </c>
+      <c r="F398">
         <f t="shared" si="14"/>
-        <v>397</v>
-      </c>
-    </row>
-    <row r="399" spans="1:1">
+        <v>26</v>
+      </c>
+      <c r="G398" t="s">
+        <v>418</v>
+      </c>
+      <c r="H398" t="s">
+        <v>1322</v>
+      </c>
+      <c r="I398" t="s">
+        <v>1321</v>
+      </c>
+      <c r="J398" t="s">
+        <v>1021</v>
+      </c>
+      <c r="K398">
+        <v>6203215211</v>
+      </c>
+      <c r="L398" t="s">
+        <v>21</v>
+      </c>
+      <c r="M398" t="s">
+        <v>21</v>
+      </c>
+      <c r="N398" t="s">
+        <v>1320</v>
+      </c>
+    </row>
+    <row r="399" spans="1:14">
       <c r="A399">
+        <f t="shared" si="15"/>
+        <v>398</v>
+      </c>
+      <c r="B399" t="s">
+        <v>38</v>
+      </c>
+      <c r="C399" t="s">
+        <v>15</v>
+      </c>
+      <c r="D399" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E399" t="s">
+        <v>16</v>
+      </c>
+      <c r="F399">
         <f t="shared" si="14"/>
-        <v>398</v>
-      </c>
-    </row>
-    <row r="400" spans="1:1">
+        <v>27</v>
+      </c>
+      <c r="G399" t="s">
+        <v>418</v>
+      </c>
+      <c r="H399" t="s">
+        <v>1323</v>
+      </c>
+      <c r="I399" t="s">
+        <v>19</v>
+      </c>
+      <c r="J399" t="s">
+        <v>1324</v>
+      </c>
+      <c r="K399">
+        <v>7004730828</v>
+      </c>
+      <c r="L399" t="s">
+        <v>21</v>
+      </c>
+      <c r="M399" t="s">
+        <v>21</v>
+      </c>
+      <c r="N399" t="s">
+        <v>1305</v>
+      </c>
+    </row>
+    <row r="400" spans="1:14">
       <c r="A400">
+        <f t="shared" si="15"/>
+        <v>399</v>
+      </c>
+      <c r="B400" t="s">
+        <v>1326</v>
+      </c>
+      <c r="C400" t="s">
+        <v>76</v>
+      </c>
+      <c r="D400" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E400" t="s">
+        <v>16</v>
+      </c>
+      <c r="F400">
         <f t="shared" si="14"/>
-        <v>399</v>
-      </c>
-    </row>
-    <row r="401" spans="1:1">
+        <v>28</v>
+      </c>
+      <c r="G400" t="s">
+        <v>417</v>
+      </c>
+      <c r="H400" t="s">
+        <v>1325</v>
+      </c>
+      <c r="I400" t="s">
+        <v>404</v>
+      </c>
+      <c r="J400" t="s">
+        <v>405</v>
+      </c>
+      <c r="K400">
+        <v>6200016658</v>
+      </c>
+      <c r="L400" t="s">
+        <v>21</v>
+      </c>
+      <c r="M400" t="s">
+        <v>21</v>
+      </c>
+      <c r="N400" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="401" spans="1:14">
       <c r="A401">
+        <f t="shared" si="15"/>
+        <v>400</v>
+      </c>
+      <c r="B401" t="s">
+        <v>77</v>
+      </c>
+      <c r="C401" t="s">
+        <v>76</v>
+      </c>
+      <c r="D401" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E401" t="s">
+        <v>16</v>
+      </c>
+      <c r="F401">
         <f t="shared" si="14"/>
-        <v>400</v>
-      </c>
-    </row>
-    <row r="402" spans="1:1">
+        <v>29</v>
+      </c>
+      <c r="G401" t="s">
+        <v>417</v>
+      </c>
+      <c r="I401" t="s">
+        <v>1327</v>
+      </c>
+      <c r="J401" t="s">
+        <v>1160</v>
+      </c>
+      <c r="K401">
+        <v>9113125993</v>
+      </c>
+      <c r="L401" t="s">
+        <v>21</v>
+      </c>
+      <c r="M401" t="s">
+        <v>21</v>
+      </c>
+      <c r="N401" t="s">
+        <v>992</v>
+      </c>
+    </row>
+    <row r="402" spans="1:14">
       <c r="A402">
+        <f t="shared" si="15"/>
+        <v>401</v>
+      </c>
+      <c r="B402" t="s">
+        <v>167</v>
+      </c>
+      <c r="C402" t="s">
+        <v>146</v>
+      </c>
+      <c r="D402" t="s">
+        <v>1228</v>
+      </c>
+      <c r="E402" t="s">
+        <v>16</v>
+      </c>
+      <c r="F402">
         <f t="shared" si="14"/>
-        <v>401</v>
-      </c>
-    </row>
-    <row r="403" spans="1:1">
+        <v>30</v>
+      </c>
+      <c r="G402" t="s">
+        <v>1330</v>
+      </c>
+      <c r="I402" t="s">
+        <v>1329</v>
+      </c>
+      <c r="J402" t="s">
+        <v>1328</v>
+      </c>
+      <c r="K402">
+        <v>852949161</v>
+      </c>
+      <c r="L402" t="s">
+        <v>165</v>
+      </c>
+      <c r="M402" t="s">
+        <v>21</v>
+      </c>
+      <c r="N402" t="s">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="403" spans="1:14">
       <c r="A403">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>402</v>
       </c>
     </row>
-    <row r="404" spans="1:1">
+    <row r="404" spans="1:14">
       <c r="A404">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>403</v>
       </c>
     </row>
-    <row r="405" spans="1:1">
+    <row r="405" spans="1:14">
       <c r="A405">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>404</v>
       </c>
     </row>
-    <row r="406" spans="1:1">
+    <row r="406" spans="1:14">
       <c r="A406">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>405</v>
       </c>
     </row>
-    <row r="407" spans="1:1">
+    <row r="407" spans="1:14">
       <c r="A407">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>406</v>
       </c>
     </row>
-    <row r="408" spans="1:1">
+    <row r="408" spans="1:14">
       <c r="A408">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>407</v>
       </c>
     </row>
-    <row r="409" spans="1:1">
+    <row r="409" spans="1:14">
       <c r="A409">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>408</v>
       </c>
     </row>
-    <row r="410" spans="1:1">
+    <row r="410" spans="1:14">
       <c r="A410">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>409</v>
       </c>
     </row>
-    <row r="411" spans="1:1">
+    <row r="411" spans="1:14">
       <c r="A411">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>410</v>
       </c>
     </row>
-    <row r="412" spans="1:1">
+    <row r="412" spans="1:14">
       <c r="A412">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>411</v>
       </c>
     </row>
-    <row r="413" spans="1:1">
+    <row r="413" spans="1:14">
       <c r="A413">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>412</v>
       </c>
     </row>
-    <row r="414" spans="1:1">
+    <row r="414" spans="1:14">
       <c r="A414">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>413</v>
       </c>
     </row>
-    <row r="415" spans="1:1">
+    <row r="415" spans="1:14">
       <c r="A415">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>414</v>
       </c>
     </row>
-    <row r="416" spans="1:1">
+    <row r="416" spans="1:14">
       <c r="A416">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>415</v>
       </c>
     </row>
     <row r="417" spans="1:1">
       <c r="A417">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>416</v>
       </c>
     </row>
     <row r="418" spans="1:1">
       <c r="A418">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>417</v>
       </c>
     </row>
     <row r="419" spans="1:1">
       <c r="A419">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>418</v>
       </c>
     </row>
     <row r="420" spans="1:1">
       <c r="A420">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>419</v>
       </c>
     </row>
     <row r="421" spans="1:1">
       <c r="A421">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>420</v>
       </c>
     </row>
     <row r="422" spans="1:1">
       <c r="A422">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>421</v>
       </c>
     </row>
     <row r="423" spans="1:1">
       <c r="A423">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>422</v>
       </c>
     </row>
     <row r="424" spans="1:1">
       <c r="A424">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>423</v>
       </c>
     </row>
     <row r="425" spans="1:1">
       <c r="A425">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>424</v>
       </c>
     </row>
     <row r="426" spans="1:1">
       <c r="A426">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>425</v>
       </c>
     </row>
     <row r="427" spans="1:1">
       <c r="A427">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>426</v>
       </c>
     </row>
     <row r="428" spans="1:1">
       <c r="A428">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>427</v>
       </c>
     </row>
     <row r="429" spans="1:1">
       <c r="A429">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>428</v>
       </c>
     </row>
     <row r="430" spans="1:1">
       <c r="A430">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>429</v>
       </c>
     </row>
     <row r="431" spans="1:1">
       <c r="A431">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>430</v>
       </c>
     </row>
     <row r="432" spans="1:1">
       <c r="A432">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>431</v>
       </c>
     </row>
     <row r="433" spans="1:1">
       <c r="A433">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>432</v>
       </c>
     </row>
     <row r="434" spans="1:1">
       <c r="A434">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>433</v>
       </c>
     </row>
     <row r="435" spans="1:1">
       <c r="A435">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>434</v>
       </c>
     </row>
     <row r="436" spans="1:1">
       <c r="A436">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>435</v>
       </c>
     </row>
     <row r="437" spans="1:1">
       <c r="A437">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>436</v>
       </c>
     </row>
     <row r="438" spans="1:1">
       <c r="A438">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>437</v>
       </c>
     </row>
     <row r="439" spans="1:1">
       <c r="A439">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>438</v>
       </c>
     </row>

</xml_diff>